<commit_message>
Handled NPI Lists feedback
</commit_message>
<xml_diff>
--- a/src/main/resources/uploadfiles/NPIStaticList.xlsx
+++ b/src/main/resources/uploadfiles/NPIStaticList.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\psevak\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rsherkar\IdeaProjects\PulsePoint_Coding\src\main\resources\uploadfiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B61757F-F970-43AC-858E-CB0D10157FD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45BB9182-62AE-4738-8A47-5BF7889DFB87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{22F7FDF5-C1DB-47E6-950D-41040D1E77D1}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{22F7FDF5-C1DB-47E6-950D-41040D1E77D1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -410,40 +410,515 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F043F20-1601-4B0F-9793-AF17080ECA4C}">
-  <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:A101"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.109375" customWidth="1"/>
+    <col min="1" max="1" width="11.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1297279022</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>1297279037</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>1297279052</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1297279067</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>1297279082</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>1297279083</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>1297279084</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>1297279085</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>1297279086</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>1297279087</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <v>1297279088</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>1297279089</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A14">
+        <v>1297279090</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>1297279091</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A16">
+        <v>1297279092</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>1297279093</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A18">
+        <v>1297279094</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <v>1297279095</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A20">
+        <v>1297279096</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A21">
+        <v>1297279097</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A22">
+        <v>1297279098</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A23">
+        <v>1297279099</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A24">
+        <v>1297279100</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A25">
+        <v>1297279101</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A26">
+        <v>1297279102</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A27">
+        <v>1297279103</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A28">
+        <v>1297279104</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A29">
+        <v>1297279105</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A30">
+        <v>1297279106</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A31">
+        <v>1297279107</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A32">
+        <v>1297279108</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A33">
+        <v>1297279109</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A34">
+        <v>1297279110</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A35">
+        <v>1297279111</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A36">
+        <v>1297279112</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A37">
+        <v>1297279113</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A38">
+        <v>1297279114</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A39">
+        <v>1297279115</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A40">
+        <v>1297279116</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A41">
+        <v>1297279117</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A42">
+        <v>1297279118</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A43">
+        <v>1297279119</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A44">
+        <v>1297279120</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A45">
+        <v>1297279121</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A46">
+        <v>1297279122</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A47">
+        <v>1297279123</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A48">
+        <v>1297279124</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A49">
+        <v>1297279125</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A50">
+        <v>1297279126</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A51">
+        <v>1297279127</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A52">
+        <v>1297279128</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A53">
+        <v>1297279129</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A54">
+        <v>1297279130</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A55">
+        <v>1297279131</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A56">
+        <v>1297279132</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A57">
+        <v>1297279133</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A58">
+        <v>1297279134</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A59">
+        <v>1297279135</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A60">
+        <v>1297279136</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A61">
+        <v>1297279137</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A62">
+        <v>1297279138</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A63">
+        <v>1297279139</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A64">
+        <v>1297279140</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A65">
+        <v>1297279141</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A66">
+        <v>1297279142</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A67">
+        <v>1297279143</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A68">
+        <v>1297279144</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A69">
+        <v>1297279145</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A70">
+        <v>1297279146</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A71">
+        <v>1297279147</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A72">
+        <v>1297279148</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A73">
+        <v>1297279149</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A74">
+        <v>1297279150</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A75">
+        <v>1297279151</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A76">
+        <v>1297279152</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A77">
+        <v>1297279153</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A78">
+        <v>1297279154</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A79">
+        <v>1297279155</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A80">
+        <v>1297279156</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A81">
+        <v>1297279157</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A82">
+        <v>1297279158</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A83">
+        <v>1297279159</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A84">
+        <v>1297279160</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A85">
+        <v>1297279161</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A86">
+        <v>1297279162</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A87">
+        <v>1297279163</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A88">
+        <v>1297279164</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A89">
+        <v>1297279165</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A90">
+        <v>1297279166</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A91">
+        <v>1297279167</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A92">
+        <v>1297279168</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A93">
+        <v>1297279169</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A94">
+        <v>1297279170</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A95">
+        <v>1297279171</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A96">
+        <v>1297279172</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A97">
+        <v>1297279173</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A98">
+        <v>1297279174</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A99">
+        <v>1297279175</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A100">
+        <v>1297279176</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A101">
+        <v>1297279177</v>
       </c>
     </row>
   </sheetData>

</xml_diff>